<commit_message>
Review pack: rebuilt with the new Primary quiz lines
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/review/language_review.xlsx
+++ b/docs/review/language_review.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F249"/>
+  <dimension ref="A1:F251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6277,9 +6277,57 @@
       <c r="E249" s="4" t="inlineStr"/>
       <c r="F249" s="4" t="inlineStr"/>
     </row>
+    <row r="250">
+      <c r="A250" s="4" t="inlineStr">
+        <is>
+          <t>Spoken lines</t>
+        </is>
+      </c>
+      <c r="B250" s="4" t="inlineStr">
+        <is>
+          <t>Practice quiz</t>
+        </is>
+      </c>
+      <c r="C250" s="4" t="inlineStr">
+        <is>
+          <t>In primary classes, tap your answer. Voice answers come later.</t>
+        </is>
+      </c>
+      <c r="D250" s="4" t="inlineStr">
+        <is>
+          <t>A azuzuwan firamare, taɓa amsarka. Amsa da murya za ta zo daga baya.</t>
+        </is>
+      </c>
+      <c r="E250" s="4" t="inlineStr"/>
+      <c r="F250" s="4" t="inlineStr"/>
+    </row>
+    <row r="251">
+      <c r="A251" s="4" t="inlineStr">
+        <is>
+          <t>Spoken lines</t>
+        </is>
+      </c>
+      <c r="B251" s="4" t="inlineStr">
+        <is>
+          <t>Practice quiz</t>
+        </is>
+      </c>
+      <c r="C251" s="4" t="inlineStr">
+        <is>
+          <t>In primary classes, tap or click your answer, or press {letters} on your keyboard.</t>
+        </is>
+      </c>
+      <c r="D251" s="4" t="inlineStr">
+        <is>
+          <t>A azuzuwan firamare, taɓa ko danna amsarka, ko ka danna {letters} a kan madannai.</t>
+        </is>
+      </c>
+      <c r="E251" s="4" t="inlineStr"/>
+      <c r="F251" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="E2:E249" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E251" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"yes,fix"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6293,7 +6341,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F260"/>
+  <dimension ref="A1:F262"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -12276,9 +12324,57 @@
       <c r="E260" s="4" t="inlineStr"/>
       <c r="F260" s="4" t="inlineStr"/>
     </row>
+    <row r="261">
+      <c r="A261" s="4" t="inlineStr">
+        <is>
+          <t>Spoken lines</t>
+        </is>
+      </c>
+      <c r="B261" s="4" t="inlineStr">
+        <is>
+          <t>Practice quiz</t>
+        </is>
+      </c>
+      <c r="C261" s="4" t="inlineStr">
+        <is>
+          <t>In primary classes, tap your answer. Voice answers come later.</t>
+        </is>
+      </c>
+      <c r="D261" s="4" t="inlineStr">
+        <is>
+          <t>Ní kíláàsì alákọ̀ọ́bẹ̀rẹ̀, tẹ ìdáhùn rẹ. Ìdáhùn pẹ̀lú ohùn yóò dé lẹ́yìn náà.</t>
+        </is>
+      </c>
+      <c r="E261" s="4" t="inlineStr"/>
+      <c r="F261" s="4" t="inlineStr"/>
+    </row>
+    <row r="262">
+      <c r="A262" s="4" t="inlineStr">
+        <is>
+          <t>Spoken lines</t>
+        </is>
+      </c>
+      <c r="B262" s="4" t="inlineStr">
+        <is>
+          <t>Practice quiz</t>
+        </is>
+      </c>
+      <c r="C262" s="4" t="inlineStr">
+        <is>
+          <t>In primary classes, tap or click your answer, or press {letters} on your keyboard.</t>
+        </is>
+      </c>
+      <c r="D262" s="4" t="inlineStr">
+        <is>
+          <t>Ní kíláàsì alákọ̀ọ́bẹ̀rẹ̀, tẹ tàbí kílíkì ìdáhùn rẹ, tàbí tẹ {letters} lórí kíbọ́ọ̀dù rẹ.</t>
+        </is>
+      </c>
+      <c r="E262" s="4" t="inlineStr"/>
+      <c r="F262" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="E2:E260" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E262" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"yes,fix"</formula1>
     </dataValidation>
   </dataValidations>
@@ -12292,7 +12388,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F225"/>
+  <dimension ref="A1:F227"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -17575,9 +17671,57 @@
       <c r="E225" s="4" t="inlineStr"/>
       <c r="F225" s="4" t="inlineStr"/>
     </row>
+    <row r="226">
+      <c r="A226" s="4" t="inlineStr">
+        <is>
+          <t>Spoken lines</t>
+        </is>
+      </c>
+      <c r="B226" s="4" t="inlineStr">
+        <is>
+          <t>Practice quiz</t>
+        </is>
+      </c>
+      <c r="C226" s="4" t="inlineStr">
+        <is>
+          <t>In primary classes, tap your answer. Voice answers come later.</t>
+        </is>
+      </c>
+      <c r="D226" s="4" t="inlineStr">
+        <is>
+          <t>Na klaasị praịmarị, pịa azịza gị. Ịza n'olu ga-abịa ma emechaa.</t>
+        </is>
+      </c>
+      <c r="E226" s="4" t="inlineStr"/>
+      <c r="F226" s="4" t="inlineStr"/>
+    </row>
+    <row r="227">
+      <c r="A227" s="4" t="inlineStr">
+        <is>
+          <t>Spoken lines</t>
+        </is>
+      </c>
+      <c r="B227" s="4" t="inlineStr">
+        <is>
+          <t>Practice quiz</t>
+        </is>
+      </c>
+      <c r="C227" s="4" t="inlineStr">
+        <is>
+          <t>In primary classes, tap or click your answer, or press {letters} on your keyboard.</t>
+        </is>
+      </c>
+      <c r="D227" s="4" t="inlineStr">
+        <is>
+          <t>Na klaasị praịmarị, pịa ma ọ bụ kpịa azịza gị, ma ọ bụ pịa {letters} na kiiboodu gị.</t>
+        </is>
+      </c>
+      <c r="E227" s="4" t="inlineStr"/>
+      <c r="F227" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="E2:E225" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E227" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"yes,fix"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>